<commit_message>
Update account page layout
</commit_message>
<xml_diff>
--- a/exports/MAXKY_SALES.xlsx
+++ b/exports/MAXKY_SALES.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -518,7 +518,7 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="E4" s="6" t="n">
-        <v>417</v>
+        <v>297</v>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B5" s="6" t="n">
-        <v>290</v>
+        <v>170</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
@@ -614,53 +614,53 @@
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>2026-08-22 01:43:16</t>
+          <t>2026-08-22 20:38:01</t>
         </is>
       </c>
       <c r="B10" s="9" t="inlineStr">
         <is>
-          <t>งานแต่ง</t>
+          <t>งานพระบาท</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>เสื้อยืด</t>
+          <t>เสื้อกีฬา</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
         <is>
-          <t>XL</t>
+          <t>L</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>99</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>2026-08-22 01:43:16</t>
+          <t>2026-08-22 20:38:01</t>
         </is>
       </c>
       <c r="B11" s="9" t="inlineStr">
         <is>
-          <t>งานแต่ง</t>
+          <t>งานพระบาท</t>
         </is>
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>เสื้อยืด</t>
+          <t>เสื้อกีฬา</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>M</t>
         </is>
       </c>
       <c r="E11" s="10" t="n">
@@ -676,63 +676,32 @@
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>2026-08-22 01:43:08</t>
+          <t>2026-08-22 20:38:01</t>
         </is>
       </c>
       <c r="B12" s="9" t="inlineStr">
         <is>
-          <t>งานแต่ง</t>
+          <t>งานพระบาท</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>เสื้อยืด</t>
+          <t>เสื้อกีฬา</t>
         </is>
       </c>
       <c r="D12" s="9" t="inlineStr">
         <is>
-          <t>3XL</t>
+          <t>S</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>120</v>
+        <v>99</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-22 01:43:08</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>งานแต่ง</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>เสื้อยืด</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>65</v>
-      </c>
-      <c r="F13" s="10" t="n">
-        <v>99</v>
-      </c>
-      <c r="G13" s="10" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>